<commit_message>
make glossary AI ready, add md and json buttons in terms
</commit_message>
<xml_diff>
--- a/exports/xlsx/terms_definition_2.xlsx
+++ b/exports/xlsx/terms_definition_2.xlsx
@@ -456,63 +456,59 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Geolocating</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>- base
-description: Value and possibly Uncertainty of a Trait of a specific Entity.</t>
+          <t>- core
+description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Scientific or technical measurements, values calculated therefrom, observations, or facts that can be represented by numbers, tables, graphs, models, text, or symbols which are used as a basis for reasoning and further calculation.</t>
+          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Entity</t>
+          <t>Instrument Data</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>- base
-description: Something that has separate and distinct existence and objective or conceptual reality.</t>
+          <t>- core
+description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
+          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ancillary Data</t>
+          <t>Auxiliary Data</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -524,352 +520,356 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Data other than instrument measurements, originating in the instrument itself or from the satellite, required to perform processing of the Data. Includes orbit Data, attitude Data, time Information, and spacecraft engineering Data, Calibration Data, Data quality Information, and Data from other instruments or earth system models.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>- CEOS-ARD PFS template 20220302</t>
+          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
+- EO Data Stewardship Glossary</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Verification</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>- core
-description: Provision of objective evidence that a given item fulfils specified requirements.</t>
+description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Evaluation of whether or not a product, service, or system complies with a regulation requirement, specification, or imposed condition. Often an internal Process.</t>
+          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>- EU-US Land Imaging EO Collaboration</t>
+          <t>- VIM?, modified</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Geolocating</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>- core
-description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
+          <t>- base
+description: Something that has separate and distinct existence and objective or conceptual reality.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
+          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Georectifying</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+description: Correcting for positional displacement with respect to the surface of the Earth.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Orthorectifying</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
+          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- KCEO</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Auxiliary Data</t>
+          <t>Uncertainty</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
+          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
+          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
+- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
-- EO Data Stewardship Glossary</t>
+          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>- core
+description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Process aimed at verifying that the specified requirements are achieved or compliant. Involves comparing mission products with representative reference data, considering various observation conditions, ensuring the quality and traceability of the reference data used.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>- BIPM; QA4EO; ESA?, modified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>- base
+description: Value and possibly Uncertainty of a Trait of a specific Entity.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Scientific or technical measurements, values calculated therefrom, observations, or facts that can be represented by numbers, tables, graphs, models, text, or symbols which are used as a basis for reasoning and further calculation.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>- base
 description: Property having a magnitude that can be expressed as a number from a continuous and contiguous range and a reference.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Property whose instances can be compared by ratio or only by order.</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>- gEOGlos (VIM4 Notes omitted)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Characteristic</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>- base
-- approved</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Abstraction of a Property of an Object or of a set of objects.</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>- Characteristics are used for describing Concepts.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Validation</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>- core
-description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
-        </is>
-      </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Process aimed at verifying that the specified requirements are achieved or compliant. Involves comparing mission products with representative reference data, considering various observation conditions, ensuring the quality and traceability of the reference data used.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
-        </is>
-      </c>
+          <t>Property whose instances can be compared by ratio or only by order.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>- BIPM; QA4EO; ESA?, modified</t>
+          <t>- gEOGlos (VIM4 Notes omitted)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Verification</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>- core
-description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
+description: Provision of objective evidence that a given item fulfils specified requirements.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
+          <t>Evaluation of whether or not a product, service, or system complies with a regulation requirement, specification, or imposed condition. Often an internal Process.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>- VIM?, modified</t>
+          <t>- EU-US Land Imaging EO Collaboration</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Georectifying</t>
+          <t>Baseline</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>- core
-description: Correcting for positional displacement with respect to the surface of the Earth.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Orthorectifying</t>
-        </is>
-      </c>
+- approved</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
+          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>- KCEO</t>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Ancillary Data</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>- core
-description: Entity (person, organization, institution, etc.) that is requesting data or information with certain characteristics described by needs and/or requirements.</t>
+- approved</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>External person, institution or system that consumes provided services.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
-        </is>
-      </c>
+          <t>Data other than instrument measurements, originating in the instrument itself or from the satellite, required to perform processing of the Data. Includes orbit Data, attitude Data, time Information, and spacecraft engineering Data, Calibration Data, Data quality Information, and Data from other instruments or earth system models.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>- EO Data Stewardship Glossary</t>
+          <t>- CEOS-ARD PFS template 20220302</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Uncertainty</t>
+          <t>User</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
           <t>- core
-description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
+description: Entity (person, organization, institution, etc.) that is requesting data or information with certain characteristics described by needs and/or requirements.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
+          <t>External person, institution or system that consumes provided services.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
-- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
+          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
+          <t>- EO Data Stewardship Glossary</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Instrument Data</t>
+          <t>Characteristic</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>- core
-description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
+          <t>- base
+- approved</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Abstraction of a Property of an Object or of a set of objects.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>- Characteristics are used for describing Concepts.</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
+          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add Data Access page, WIP disclaimer banner, and updated exports
- New docs/ai-readiness.md page covering all data access patterns (JSON, Parquet, XLSX, llms.txt, MCP server, per-term endpoints)
- Site-wide announcement bar with WIP disclaimer (session-only dismissal via client module)
- Disclaimer added to README.md
- Updated glossary exports

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/xlsx/terms_definition_2.xlsx
+++ b/exports/xlsx/terms_definition_2.xlsx
@@ -456,63 +456,59 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Geolocating</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>- base
-description: Value and possibly Uncertainty of a Trait of a specific Entity.</t>
+          <t>- core
+description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Scientific or technical measurements, values calculated therefrom, observations, or facts that can be represented by numbers, tables, graphs, models, text, or symbols which are used as a basis for reasoning and further calculation.</t>
+          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Entity</t>
+          <t>Instrument Data</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>- base
-description: Something that has separate and distinct existence and objective or conceptual reality.</t>
+          <t>- core
+description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
+          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ancillary Data</t>
+          <t>Auxiliary Data</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -524,352 +520,356 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Data other than instrument measurements, originating in the instrument itself or from the satellite, required to perform processing of the Data. Includes orbit Data, attitude Data, time Information, and spacecraft engineering Data, Calibration Data, Data quality Information, and Data from other instruments or earth system models.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>- CEOS-ARD PFS template 20220302</t>
+          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
+- EO Data Stewardship Glossary</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Verification</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>- core
-description: Provision of objective evidence that a given item fulfils specified requirements.</t>
+description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Evaluation of whether or not a product, service, or system complies with a regulation requirement, specification, or imposed condition. Often an internal Process.</t>
+          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>- EU-US Land Imaging EO Collaboration</t>
+          <t>- VIM?, modified</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Geolocating</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>- core
-description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
+          <t>- base
+description: Something that has separate and distinct existence and objective or conceptual reality.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
+          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Georectifying</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+description: Correcting for positional displacement with respect to the surface of the Earth.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Orthorectifying</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
+          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- KCEO</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Auxiliary Data</t>
+          <t>Uncertainty</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
+          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
+          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
+- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
-- EO Data Stewardship Glossary</t>
+          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>- core
+description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Process aimed at verifying that the specified requirements are achieved or compliant. Involves comparing mission products with representative reference data, considering various observation conditions, ensuring the quality and traceability of the reference data used.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>- BIPM; QA4EO; ESA?, modified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>- base
+description: Value and possibly Uncertainty of a Trait of a specific Entity.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Scientific or technical measurements, values calculated therefrom, observations, or facts that can be represented by numbers, tables, graphs, models, text, or symbols which are used as a basis for reasoning and further calculation.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>- base
 description: Property having a magnitude that can be expressed as a number from a continuous and contiguous range and a reference.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Property whose instances can be compared by ratio or only by order.</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>- gEOGlos (VIM4 Notes omitted)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Characteristic</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>- base
-- approved</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Abstraction of a Property of an Object or of a set of objects.</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>- Characteristics are used for describing Concepts.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Validation</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>- core
-description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
-        </is>
-      </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Process aimed at verifying that the specified requirements are achieved or compliant. Involves comparing mission products with representative reference data, considering various observation conditions, ensuring the quality and traceability of the reference data used.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
-        </is>
-      </c>
+          <t>Property whose instances can be compared by ratio or only by order.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>- BIPM; QA4EO; ESA?, modified</t>
+          <t>- gEOGlos (VIM4 Notes omitted)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Verification</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>- core
-description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
+description: Provision of objective evidence that a given item fulfils specified requirements.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
+          <t>Evaluation of whether or not a product, service, or system complies with a regulation requirement, specification, or imposed condition. Often an internal Process.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>- VIM?, modified</t>
+          <t>- EU-US Land Imaging EO Collaboration</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Georectifying</t>
+          <t>Baseline</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>- core
-description: Correcting for positional displacement with respect to the surface of the Earth.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Orthorectifying</t>
-        </is>
-      </c>
+- approved</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
+          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>- KCEO</t>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Ancillary Data</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>- core
-description: Entity (person, organization, institution, etc.) that is requesting data or information with certain characteristics described by needs and/or requirements.</t>
+- approved</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>External person, institution or system that consumes provided services.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
-        </is>
-      </c>
+          <t>Data other than instrument measurements, originating in the instrument itself or from the satellite, required to perform processing of the Data. Includes orbit Data, attitude Data, time Information, and spacecraft engineering Data, Calibration Data, Data quality Information, and Data from other instruments or earth system models.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>- EO Data Stewardship Glossary</t>
+          <t>- CEOS-ARD PFS template 20220302</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Uncertainty</t>
+          <t>User</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
           <t>- core
-description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
+description: Entity (person, organization, institution, etc.) that is requesting data or information with certain characteristics described by needs and/or requirements.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
+          <t>External person, institution or system that consumes provided services.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
-- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
+          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
+          <t>- EO Data Stewardship Glossary</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Instrument Data</t>
+          <t>Characteristic</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>- core
-description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
+          <t>- base
+- approved</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Abstraction of a Property of an Object or of a set of objects.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>- Characteristics are used for describing Concepts.</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
+          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: update Node.js from 20 to 22 (current LTS)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/xlsx/terms_definition_2.xlsx
+++ b/exports/xlsx/terms_definition_2.xlsx
@@ -456,63 +456,59 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Geolocating</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>- base
-description: Value and possibly Uncertainty of a Trait of a specific Entity.</t>
+          <t>- core
+description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Scientific or technical measurements, values calculated therefrom, observations, or facts that can be represented by numbers, tables, graphs, models, text, or symbols which are used as a basis for reasoning and further calculation.</t>
+          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Entity</t>
+          <t>Instrument Data</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>- base
-description: Something that has separate and distinct existence and objective or conceptual reality.</t>
+          <t>- core
+description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
+          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ancillary Data</t>
+          <t>Auxiliary Data</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -524,352 +520,356 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Data other than instrument measurements, originating in the instrument itself or from the satellite, required to perform processing of the Data. Includes orbit Data, attitude Data, time Information, and spacecraft engineering Data, Calibration Data, Data quality Information, and Data from other instruments or earth system models.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>- CEOS-ARD PFS template 20220302</t>
+          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
+- EO Data Stewardship Glossary</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Verification</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>- core
-description: Provision of objective evidence that a given item fulfils specified requirements.</t>
+description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Evaluation of whether or not a product, service, or system complies with a regulation requirement, specification, or imposed condition. Often an internal Process.</t>
+          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>- EU-US Land Imaging EO Collaboration</t>
+          <t>- VIM?, modified</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Geolocating</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>- core
-description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
+          <t>- base
+description: Something that has separate and distinct existence and objective or conceptual reality.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
+          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Georectifying</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+description: Correcting for positional displacement with respect to the surface of the Earth.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Orthorectifying</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
+          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- KCEO</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Auxiliary Data</t>
+          <t>Uncertainty</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
+          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
+          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
+- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
-- EO Data Stewardship Glossary</t>
+          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>- core
+description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Process aimed at verifying that the specified requirements are achieved or compliant. Involves comparing mission products with representative reference data, considering various observation conditions, ensuring the quality and traceability of the reference data used.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>- BIPM; QA4EO; ESA?, modified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>- base
+description: Value and possibly Uncertainty of a Trait of a specific Entity.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Scientific or technical measurements, values calculated therefrom, observations, or facts that can be represented by numbers, tables, graphs, models, text, or symbols which are used as a basis for reasoning and further calculation.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>- base
 description: Property having a magnitude that can be expressed as a number from a continuous and contiguous range and a reference.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Property whose instances can be compared by ratio or only by order.</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>- gEOGlos (VIM4 Notes omitted)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Characteristic</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>- base
-- approved</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Abstraction of a Property of an Object or of a set of objects.</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>- Characteristics are used for describing Concepts.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Validation</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>- core
-description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
-        </is>
-      </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Process aimed at verifying that the specified requirements are achieved or compliant. Involves comparing mission products with representative reference data, considering various observation conditions, ensuring the quality and traceability of the reference data used.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
-        </is>
-      </c>
+          <t>Property whose instances can be compared by ratio or only by order.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>- BIPM; QA4EO; ESA?, modified</t>
+          <t>- gEOGlos (VIM4 Notes omitted)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Verification</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>- core
-description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
+description: Provision of objective evidence that a given item fulfils specified requirements.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
+          <t>Evaluation of whether or not a product, service, or system complies with a regulation requirement, specification, or imposed condition. Often an internal Process.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>- VIM?, modified</t>
+          <t>- EU-US Land Imaging EO Collaboration</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Georectifying</t>
+          <t>Baseline</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>- core
-description: Correcting for positional displacement with respect to the surface of the Earth.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Orthorectifying</t>
-        </is>
-      </c>
+- approved</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
+          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>- KCEO</t>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Ancillary Data</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>- core
-description: Entity (person, organization, institution, etc.) that is requesting data or information with certain characteristics described by needs and/or requirements.</t>
+- approved</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>External person, institution or system that consumes provided services.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
-        </is>
-      </c>
+          <t>Data other than instrument measurements, originating in the instrument itself or from the satellite, required to perform processing of the Data. Includes orbit Data, attitude Data, time Information, and spacecraft engineering Data, Calibration Data, Data quality Information, and Data from other instruments or earth system models.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>- EO Data Stewardship Glossary</t>
+          <t>- CEOS-ARD PFS template 20220302</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Uncertainty</t>
+          <t>User</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
           <t>- core
-description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
+description: Entity (person, organization, institution, etc.) that is requesting data or information with certain characteristics described by needs and/or requirements.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
+          <t>External person, institution or system that consumes provided services.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
-- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
+          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
+          <t>- EO Data Stewardship Glossary</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Instrument Data</t>
+          <t>Characteristic</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>- core
-description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
+          <t>- base
+- approved</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Abstraction of a Property of an Object or of a set of objects.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>- Characteristics are used for describing Concepts.</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
+          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: display clickable tag badges on term pages
Swizzle DocItem/Content to render frontmatter tags as color-coded
badges right below the heading. Badges link to their tag pages
(e.g. /tags/to-be-approved). Add CSS flex ordering to position
badges between h1 and content.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/xlsx/terms_definition_2.xlsx
+++ b/exports/xlsx/terms_definition_2.xlsx
@@ -456,431 +456,431 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Geolocating</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Instrument Data</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>- core
+  - to be approved
+description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Auxiliary Data</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
+- EO Data Stewardship Glossary</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>- core
+- to be discussed
+description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>- VIM?, modified</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>- base
+- to be approved
+description: Something that has separate and distinct existence and objective or conceptual reality.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Georectifying</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>- core
+  - to be discussed
+description: Correcting for positional displacement with respect to the surface of the Earth.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Orthorectifying</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>- KCEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Uncertainty</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
+- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Process aimed at verifying that the specified requirements are achieved or compliant. Involves comparing mission products with representative reference data, considering various observation conditions, ensuring the quality and traceability of the reference data used.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>- BIPM; QA4EO; ESA?, modified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>- base
 - to be approved
 description: Value and possibly Uncertainty of a Trait of a specific Entity.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
         <is>
           <t>Scientific or technical measurements, values calculated therefrom, observations, or facts that can be represented by numbers, tables, graphs, models, text, or symbols which are used as a basis for reasoning and further calculation.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
         <is>
           <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Entity</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>- base
-- to be approved
-description: Something that has separate and distinct existence and objective or conceptual reality.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Ancillary Data</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Data other than instrument measurements, originating in the instrument itself or from the satellite, required to perform processing of the Data. Includes orbit Data, attitude Data, time Information, and spacecraft engineering Data, Calibration Data, Data quality Information, and Data from other instruments or earth system models.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>- CEOS-ARD PFS template 20220302</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Verification</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved
-description: Provision of objective evidence that a given item fulfils specified requirements.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Evaluation of whether or not a product, service, or system complies with a regulation requirement, specification, or imposed condition. Often an internal Process.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>- EU-US Land Imaging EO Collaboration</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Geolocating</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved
-description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Auxiliary Data</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
-- EO Data Stewardship Glossary</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>- base
 - to be approved
 description: Property having a magnitude that can be expressed as a number from a continuous and contiguous range and a reference.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Property whose instances can be compared by ratio or only by order.</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>- gEOGlos (VIM4 Notes omitted)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Characteristic</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>- base
-- to be discussed</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Abstraction of a Property of an Object or of a set of objects.</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>- Characteristics are used for describing Concepts.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Validation</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved
-description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
-        </is>
-      </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Process aimed at verifying that the specified requirements are achieved or compliant. Involves comparing mission products with representative reference data, considering various observation conditions, ensuring the quality and traceability of the reference data used.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
-        </is>
-      </c>
+          <t>Property whose instances can be compared by ratio or only by order.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>- BIPM; QA4EO; ESA?, modified</t>
+          <t>- gEOGlos (VIM4 Notes omitted)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Verification</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>- core
-- to be discussed
-description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
+- to be approved
+description: Provision of objective evidence that a given item fulfils specified requirements.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
+          <t>Evaluation of whether or not a product, service, or system complies with a regulation requirement, specification, or imposed condition. Often an internal Process.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>- VIM?, modified</t>
+          <t>- EU-US Land Imaging EO Collaboration</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Georectifying</t>
+          <t>Baseline</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>- core
-  - to be discussed
-description: Correcting for positional displacement with respect to the surface of the Earth.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Orthorectifying</t>
-        </is>
-      </c>
+- to be approved</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
+          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>- KCEO</t>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Ancillary Data</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Data other than instrument measurements, originating in the instrument itself or from the satellite, required to perform processing of the Data. Includes orbit Data, attitude Data, time Information, and spacecraft engineering Data, Calibration Data, Data quality Information, and Data from other instruments or earth system models.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>- CEOS-ARD PFS template 20220302</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>User</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>- core
 - to be approved
 description: Entity (person, organization, institution, etc.) that is requesting data or information with certain characteristics described by needs and/or requirements.</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>External person, institution or system that consumes provided services.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>- EO Data Stewardship Glossary</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Uncertainty</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>- core
-- to be approved
-description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
-        </is>
-      </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
+          <t>External person, institution or system that consumes provided services.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
-- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
+          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
+          <t>- EO Data Stewardship Glossary</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Instrument Data</t>
+          <t>Characteristic</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>- core
-  - to be approved
-description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
+          <t>- base
+- to be discussed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Abstraction of a Property of an Object or of a set of objects.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>- Characteristics are used for describing Concepts.</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
+          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: ingest 432 CalVal portal terms into glossary (#10)
Systematic ingest of the CEOS CalVal glossary (calvalportal.ceos.org).
509 total terms (was 151): 358 new files, 37 existing terms updated.
Definitions deduplicated, cleaned, and rewritten for glossary standards.
Terms tagged with calval ingest provenance and CEOS working groups
(WGCV, WGISS, WGClimate). Added tag UI support (badges, colors,
overview page).

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/xlsx/terms_definition_2.xlsx
+++ b/exports/xlsx/terms_definition_2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,161 +456,178 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Geolocating</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>- base
-- to be approved
-description: Value and possibly Uncertainty of a Trait of a specific Entity.</t>
+          <t>- core
+- to be approved</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Scientific or technical measurements, values calculated therefrom, observations, or facts that can be represented by numbers, tables, graphs, models, text, or symbols which are used as a basis for reasoning and further calculation.</t>
+          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Entity</t>
+          <t>Instrument Data</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>- base
-- to be approved
-description: Something that has separate and distinct existence and objective or conceptual reality.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>- core
+- to be approved
+- calval ingest
+- WGCV
+- WGClimate</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sensor Data, Sensor Data Record</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
+          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ancillary Data</t>
+          <t>Auxiliary Data</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>- core
-- to be approved</t>
+- to be approved
+- calval ingest
+- WGCV
+- WGClimate</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Data other than instrument measurements, originating in the instrument itself or from the satellite, required to perform processing of the Data. Includes orbit Data, attitude Data, time Information, and spacecraft engineering Data, Calibration Data, Data quality Information, and Data from other instruments or earth system models.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>- CEOS-ARD PFS template 20220302</t>
+          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
+- EO Data Stewardship Glossary</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Verification</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>- core
 - to be approved
-description: Provision of objective evidence that a given item fulfils specified requirements.</t>
+- calval ingest
+- WGCV
+- WGClimate</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Evaluation of whether or not a product, service, or system complies with a regulation requirement, specification, or imposed condition. Often an internal Process.</t>
+          <t>Output of an organization distributable to users without transaction, derived from instrument data via processing with ancillary data, and may include metadata and browse images.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>- EU-US Land Imaging EO Collaboration</t>
+          <t>- ISO:9000 [ [RD7](https://www.iso.org/standard/45481.html) ]
+- RD7: ISO 9000:2015(en), Quality management systems - Fundamentals and vocabulary
+- [CEOS EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- NESDIS Data Management Lexicon and Related Terms</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Geolocating</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
           <t>- core
-- to be approved
-description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
+- to be discussed</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Determination of the geographic location of a feature of two or more dimensions.</t>
+          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>- ISO 19130-1:2018, 3.36 ('geopositioning'), modified</t>
+          <t>- VIM?, modified</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>- core
+          <t>- base
 - to be approved</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
+          <t>Government or business organization that is formed to conduct business or represent the government of the day.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>CEOS Entities include Working Groups, Virtual Constellations, etc.</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
@@ -620,267 +637,937 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Auxiliary Data</t>
+          <t>Collection</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>- core
-- to be approved</t>
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Data required to perform processing of Sensor Data which is not obtained from the Sensor itself. Includes: (a) Data provided by the spacecraft (e.g. orbit Position and velocity, attitude, instrument house-keeping Data, on-board time); (b) Data not available from on-board sources.</t>
+          <t>Grouping of environmental data or products sharing common characteristics, represented by a single metadata record and consisting of one or more granules; also referred to as a dataset.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>For EnMAP, this includes (a) orbit files, attitude files, Calibration Data, instrument house-keeping Data; (b) atmospheric parameters, reference images.</t>
+          <t>Note that in these definitions of “collection” and “granule” that a collection is the minimum citable unit of data, akin to a journal article. This approach helps align data citation and publication with the much more mature practices surrounding journal article publication. In this alignment, granules can be thought of as the words in that article. This functional definition allows for flexibility as well; just as current science domains have their own standards for what qualifies as a minimally citable body of work that can go into a single journal article, different data domains across NOAA can do the same and determine what makes sense to go into one of their collections. If NOAA should ever reach a more detailed definition, adjustments can be made to align the collection metadata with that new definition.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>- ENMAP Glossary of Terms, https://www.enmap.org/Data/doc/EnMAP_Terms.pdf, 20210624
-- EO Data Stewardship Glossary</t>
+          <t>- [CEOS/WGISS/DSIG/GLOS](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- [ESA PDGS Glossary, PGSI-GSEG-EOPG-LI-13-0033 (MM-PDGS Glossary Issue 2.0_forReview.docx)](https://calvalportal.ceos.org/web/guest/t-d_wiki?p_p_id=com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn&amp;p_p_lifecycle=0&amp;p_p_state=normal&amp;p_p_mode=view&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_mvcRenderCommandName=%2Fwiki%2Fedit_page&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_redirect=https%3A%2F%2Fcalvalportal.ceos.org%2Fweb%2Fguest%2Ft-d_wiki%3Fp_p_id%3Dcom_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn%26p_p_lifecycle%3D0%26p_p_state%3Dnormal%26p_p_mode%3Dview%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_mvcRenderCommandName%3D%252Fwiki%252Fview_page%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_nodeName%3DCEOS_Terms_and_Definitions%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_title%3DCollection&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_nodeId=668236&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_title=ESA+PDGS+Glossary%2C+PGSI-GSEG-EOPG-LI-13-0033+%28MM-PDGS+Glossary+Issue+2.0_forReview.docx%29)
+- This term and functional definition emerged from an ESIP session on collections and granules in the mid-2010’s.; [Reference Model for an Open Archival Information System (OAIS), Recommended Practice CCSDS 650.0-M-2, Magenta Book 2012](https://public.ccsds.org/pubs/650x0m2.pdf)
+- NESDIS Data Management Lexicon and Related Terms</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Georectifying</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>- base
-- to be approved
-description: Property having a magnitude that can be expressed as a number from a continuous and contiguous range and a reference.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>- core
+- to be discussed</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Orthorectifying</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Property whose instances can be compared by ratio or only by order.</t>
+          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>- gEOGlos (VIM4 Notes omitted)</t>
+          <t>- KCEO</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Characteristic</t>
+          <t>Uncertainty</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>- base
-- to be discussed</t>
+          <t>- core
+- to be approved
+- calval ingest
+- WGCV
+- WGISS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Abstraction of a Property of an Object or of a set of objects.</t>
+          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>- Characteristics are used for describing Concepts.</t>
+          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
+- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
+          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Standard Uncertainty</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>- core
 - to be approved
-description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
+- calval ingest
+- WGISS
+- WGCV</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Process aimed at verifying that the specified requirements are achieved or compliant. Involves comparing mission products with representative reference data, considering various observation conditions, ensuring the quality and traceability of the reference data used.</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
-        </is>
-      </c>
+          <t>Measurement uncertainty expressed as a standard deviation</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>- BIPM; QA4EO; ESA?, modified</t>
+          <t>- VIM/ISO:99 [ [RD18](https://www.bipm.org/en/publications/guides/vim.html) ]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Source Data</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>- core
-- to be discussed
-description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sort of data acquired with an Uncertainty significantly lower (quantify?) than that of the data it is being compared with.</t>
+          <t>Unprocessed data not yet transformed into meaningful information, originating from the source location in computing systems.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>- VIM?, modified</t>
+          <t>- multiple sources needs revision
+- NESDIS Data Management Lexicon and Related Terms</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Georectifying</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
           <t>- core
-  - to be discussed
-description: Correcting for positional displacement with respect to the surface of the Earth.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Orthorectifying</t>
-        </is>
-      </c>
+- to be approved
+- calval ingest
+- WGCV
+- WGClimate</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>The correction of sample locations to achieve some sort of geometric regularity, e.g., a regular 2D geographic grid.</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>Process of verifying that specified requirements are met by comparing mission products with representative reference data, ensuring quality and traceability.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>- In this part of ISO 19159, the term validation is used in a limited sense and only relates to the validation of calibration data in order to control their change over time.</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>- KCEO</t>
+          <t>- BIPM; QA4EO; ESA?, modified</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Calibration</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
           <t>- core
-- to be approved
-description: Entity (person, organization, institution, etc.) that is requesting data or information with certain characteristics described by needs and/or requirements.</t>
+- source missing
+- to be discussed
+- calval ingest
+- WGISS
+- WGCV</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>External person, institution or system that consumes provided services.</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
-        </is>
-      </c>
+          <t>Operation that establishes and applies a relation between measurement standard values and instrument indications to derive measurement results.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>- EO Data Stewardship Glossary</t>
+          <t>- (1) CEOS/ISO:19159 [RD10]: ISO/TS 19159-1:2014(en), Geographic information - Calibration and validation of remote sensing imagery sensors and data — Part 1: Optical sensors
+- (2) VIM/ISO:99 [ [RD18](https://www.bipm.org/en/publications/guides/vim.html) ]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Uncertainty</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>- core
-- to be approved
-description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
+          <t>- base
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Non-negative parameter, associated with data, which characterizes the dispersion of the values of a Trait that could reasonably be attributed to a Phenomenon by means of sensing or modelling.</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>- In case of quantitative (continuous) data the uncertainty may be, for example, a standard deviation (or a given multiple of it), or the half-width of an interval having a stated level of confidence (see e.g. Standard and Expanded Uncertainty).
-- For qualitative (categorical?) data, uncertainty may be expressed by commission and omission ('confusion matrix') or overall errors.</t>
-        </is>
-      </c>
+          <t>Scientific or technical measurements, calculated values, observations, or facts representable by numbers, tables, graphs, models, text, or symbols and used as a basis for reasoning and calculation.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>- Modified from GUM, VIM4:3.1, FIDUCEO, Notes added</t>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data
+- [CEOS/WGISS/DSIG/GLOS](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- [CEOS-WGISS Document: Auxiliary Data in the CEOS Community: Reference Guidelines Document Part 1: Current Usage (1996) accessible at wgiss.ceos.org/archive/archive.doc/ads200part1.doc](https://calvalportal.ceos.org/web/guest/t-d_wiki?p_p_id=com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn&amp;p_p_lifecycle=0&amp;p_p_state=normal&amp;p_p_mode=view&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_mvcRenderCommandName=%2Fwiki%2Fedit_page&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_redirect=https%3A%2F%2Fcalvalportal.ceos.org%2Fweb%2Fguest%2Ft-d_wiki%3Fp_p_id%3Dcom_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn%26p_p_lifecycle%3D0%26p_p_state%3Dnormal%26p_p_mode%3Dview%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_mvcRenderCommandName%3D%252Fwiki%252Fview_page%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_nodeName%3DCEOS_Terms_and_Definitions%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_title%3DData&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_nodeId=668236&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_title=CEOS-WGISS+Document%3A+Auxiliary+Data+in+the+CEOS+Community%3A+Reference+Guidelines+Document+Part+1%3A+Current+Usage+%281996%29+accessible+at+wgiss.ceos.org%2Farchive%2Farchive.doc%2Fads200part1.doc)
+- [CEOS EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf) ; [Reference Model for an Open Archival Information System (OAIS), Recommended Practice CCSDS 650.0-M-2, Magenta Book 2012](https://public.ccsds.org/pubs/650x0m2.pdf)
+- NESDIS Data Management Lexicon and Related Terms</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Instrument Data</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>- core
-  - to be approved
-description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
+          <t>- base
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Data created by an instrument including scientific measurements and any engineering or ancillary data which may be included in the data packets.</t>
+          <t>Property whose instances can be compared by ratio or only by order.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>- [EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
+          <t>- gEOGlos (VIM4 Notes omitted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Resolution</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>- core
+- to be defined
+- calval ingest
+- WGCV
+- WGClimate</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Smallest change in energy detectable and representable by the number of bits per pixel, where each bit doubles the number of possible values.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>- (1) VIM/ISO:99 [ [RD18](https://www.bipm.org/en/publications/guides/vim.html) ]; (2) NIST [RD15]; (3) MACC [RD13]
+- RD15: Prokhorov, A. V., R. U. Datla, V. P. Zakharenkov, V. Privalsky, T. W. Humpherys, and V. I. Sapritsky, Spaceborne Optoelectronic Sensors and their Radiometric Calibration. Terms and Definitions. Part 1. Calibration Techniques, Ed. by A. C. Parr and L. K. Issaev, NIST Technical Note NISTIR 7203, March 2005
+- RD13: MACC II Service Validation Protocol, Deliverable D153.1, May 2013
+- [NASA Earthdata](https://earthdata.nasa.gov/learn/backgrounders/remote-sensing)
+- NESDIS Data Management Lexicon and Related Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGCV
+- WGISS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Closeness of agreement between a measured quantity value and a true quantity value of a measurand.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>- VIM [ [RD18](https://www.bipm.org/en/publications/guides/vim.html) ], GUM [ [RD4](https://www.bipm.org/utils/common/documents/jcgm/JCGM_100_2008_E.pdf) ]
+- Definitions used in other communities
+- ACIX community
+- [Community, not standard, definition]
+- Used in the atmospheric correction community to represent the average difference between the modelled and measured quantities</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>- base
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Knowledge exchangeable in the form of data, including representation information that enables interpretation of the data.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>- [CEOS/WGISS/DSIG/GLOS](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Data describing characteristics, content, and utility of a dataset to enable search, discovery, and access management, particularly for Earth Observation resources.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>- WMO [ [RD19](http://www.bom.gov.au/wmo/quality_management.shtml) ]
+- [Reference Model for an Open Archival Information System (OAIS), Recommended Practice CCSDS 650.0-M-2, Magenta Book 2012](https://public.ccsds.org/pubs/650x0m2.pdf) ; [CEOS EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- NESDIS Data Management Lexicon and Related Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Phenomenon</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>- base
+- to be approved</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>A phenomenon is a fact or event that has
+properties
+.
+Source:
+modified after Wikipedia and The Columbia Encyclopedia 2008</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>- CEOS CalVal Portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGCV
+- WGISS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Evaluation of whether a product, service, or system complies with a regulation, specification, or imposed condition.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>- EU-US Land Imaging EO Collaboration</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>- base
+- to be discussed
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Assessable and attributable characteristic of a phenomenon, named and either observable (factual) or assigned (fictional).</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>- CEOS CalVal Portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Source data that has been processed to a common set of requirements and organised into a form that allows immediate analysis and interoperability through time and with other collections.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>- WGISS Shared Collection Lifecycle Management Principles for Earth Observation Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Subscription</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>- core
+- to be discussed
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Standing Order</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Email issued to users when new data is available from the CLASS infrastructure.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>An email provides a 'symbolic link' to new files stored in an access area. (Not sure if all 'links' are emailed or some other notification)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>- [OSGS/CLASS - NCEI/DAB](https://calvalportal.ceos.org/web/guest/t-d_wiki?p_p_id=com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn&amp;p_p_lifecycle=0&amp;p_p_state=normal&amp;p_p_mode=view&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_mvcRenderCommandName=%2Fwiki%2Fedit_page&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_redirect=https%3A%2F%2Fcalvalportal.ceos.org%2Fweb%2Fguest%2Ft-d_wiki%3Fp_p_id%3Dcom_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn%26p_p_lifecycle%3D0%26p_p_state%3Dnormal%26p_p_mode%3Dview%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_mvcRenderCommandName%3D%252Fwiki%252Fview_page%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_nodeName%3DCEOS_Terms_and_Definitions%26_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_title%3DStanding%2BOrder%2B%2528Subscription%2529&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_nodeId=668236&amp;_com_liferay_wiki_web_portlet_WikiDisplayPortlet_INSTANCE_B9cyrDcwYNcn_title=OSGS%2FCLASS+-+NCEI%2FDAB)
+- NESDIS Data Management Lexicon and Related Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Latency</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>- core
+- to be discussed
+- calval ingest
+- WGCV
+- WGClimate</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Time delay between event occurrence and use of processed data, typically within 3 hours for meteorological purposes.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>- [CEOS/WGISS/DSIG/GLOS](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Quality Indicator</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Information provided as a number, set of numbers, graph, uncertainty budget, or flag to evaluate data fitness for purpose.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>- [CEOS/WGISS/DSIG/GLOS](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Stability</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Property of a measuring instrument, whereby its metrological properties remain constant in time</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>- VIM/ISO:99 [ [RD18](https://www.bipm.org/en/publications/guides/vim.html) ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sensor</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGCV
+- WGClimate</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Device which transmits an output signal in response to a physical input stimulus as voltage. In Earth observation a distinction between passives sensors, such as radiometers, and active sensors, such as radars, is common. Earth observation sensors – or instruments – are operated from different ground-/water-based, airborne, or spaceborne platforms.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>- [CEOS/WGISS/DSIG/GLOS](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- [CEOS EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- NESDIS Data Management Lexicon and Related Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Temporal Resolution</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A time period during which data was collected or observations made, or a time period that an activity or collection is linked to intellectually or thematically, for example, 1997 to 1998; the 18th century.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>- [Australian National Data Service - Content Providers Guide - Spatial and Temporal Coverage](https://documentation.ands.org.au/display/DOC/Temporal+coverage)
+- NESDIS Data Management Lexicon and Related Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Ancillary Data</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Non-instrument data required for processing, including orbit, attitude, time, spacecraft engineering, calibration, quality, and external model data.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>- CEOS-ARD PFS template 20220302</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>External person, institution, or system consuming provided services.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>- Includes Data Access or Science and Service Exploitation Platforms provided by a payload data ground segment.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>- EO Data Stewardship Glossary
+- [CEOS/WGISS/DSIG/GLOS](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- [CEOS EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- NESDIS Data Management Lexicon and Related Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Characteristic</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>- base
+- to be discussed</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Abstraction of a Property of an Object or of a set of objects.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>- Characteristics are used for describing Concepts.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>- ISO 1087-1:2000, 3.2.4; ISO 19146:2010(E); https://www.iso.org/standard/20057.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Processes ensuring the technical and intellectual survival of space data sets and metadata over time, preserving integrity, discoverability, accessibility, and long-term reusability.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Preservation covers all processes and operations on individual or multi-mission data sets for ensuring the technical and intellectual survival of Space Data set and their metadata through time. It grants dataset integrity, its discoverability and accessibility, and facilitates its (re)-use in the long term. Preservation is one of the tasks of data curation. Examples are data record improvement and consolidation. XX</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>- [CEOS/WGISS/DSIG/GLOS](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- [Reference Model for an Open Archival Information System (OAIS), Recommended Practice CCSDS 650.0-M-2, Magenta Book 2012](https://public.ccsds.org/pubs/650x0m2.pdf) ; [CEOS EO Data Stewardship Glossary](https://ceos.org/document_management/Working_Groups/WGISS/Interest_Groups/Data_Stewardship/White_Papers/EO-DataStewardshipGlossary.pdf)
+- NESDIS Data Management Lexicon and Related Terms</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Application Programming Interface</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>- core
+- to be discussed
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>A set of functions and procedures allowing the creation of applications that access the features or data of an operating system, application, or other service.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>An application programming interface (API) is an interface that defines interactions between multiple software applications or mixed hardware-software intermediaries. It defines the kinds of calls or requests that can be made, how to make them, the data formats that should be used, the conventions to follow, etc. It can also provide extension mechanisms so that users can extend existing functionality in various ways and to varying degrees. An API can be entirely custom, specific to a component, or designed based on an industry-standard to ensure interoperability. Through information hiding, APIs enable modular programming, allowing users to use the interface independently of the implementation.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>- CEOS CalVal Portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Representativeness</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>The extent to which a set of measurements taken in a given space-time domain reflect the actual conditions in the same or different space-time domain taken on a scale appropriate for a specific application</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>- Nappo [RD14]
+- RD14: Nappo, C.J., Caneill J.Y., Furman R.W., Gifford F.A., Kaimal J.C., Kramer M.L., Lockhart T.J., Pendergast M.M, Pielke R.A., Randerson D., Shreffler J.H., and Wyngaard J.C., The Workshop on the Representativeness of Meteorological Observations, June 1981, Boulder, CO, Bull. Am. Meteorol. Soc. 63, 761-764, 1982.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Reproducibility</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>- core
+- to be approved
+- calval ingest
+- WGISS
+- WGCV</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Measurement precision under conditions including different locations, operators, measuring systems, and replicate measurements on similar objects.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>- VIM/ISO:99 [ [RD18](https://www.bipm.org/en/publications/guides/vim.html) ]</t>
         </is>
       </c>
     </row>

</xml_diff>